<commit_message>
fix(demo-data): GNDEC upload files use @gndec.test emails, so a college built from them never shares accounts with the built-in GNDEC demo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/demo-data/GNDEC/GNDEC_3_IT.xlsx
+++ b/docs/demo-data/GNDEC/GNDEC_3_IT.xlsx
@@ -4305,7 +4305,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2616001@gndec.demo</t>
+          <t>2616001@gndec.test</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2616002@gndec.demo</t>
+          <t>2616002@gndec.test</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2616003@gndec.demo</t>
+          <t>2616003@gndec.test</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2616004@gndec.demo</t>
+          <t>2616004@gndec.test</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -4413,7 +4413,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2616005@gndec.demo</t>
+          <t>2616005@gndec.test</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2616006@gndec.demo</t>
+          <t>2616006@gndec.test</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2616007@gndec.demo</t>
+          <t>2616007@gndec.test</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -4494,7 +4494,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2616008@gndec.demo</t>
+          <t>2616008@gndec.test</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -4521,7 +4521,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2616009@gndec.demo</t>
+          <t>2616009@gndec.test</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -4548,7 +4548,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2616010@gndec.demo</t>
+          <t>2616010@gndec.test</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2616011@gndec.demo</t>
+          <t>2616011@gndec.test</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2616012@gndec.demo</t>
+          <t>2616012@gndec.test</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -4629,7 +4629,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2616013@gndec.demo</t>
+          <t>2616013@gndec.test</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2616014@gndec.demo</t>
+          <t>2616014@gndec.test</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2616015@gndec.demo</t>
+          <t>2616015@gndec.test</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2616016@gndec.demo</t>
+          <t>2616016@gndec.test</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2616017@gndec.demo</t>
+          <t>2616017@gndec.test</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2616018@gndec.demo</t>
+          <t>2616018@gndec.test</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -4791,7 +4791,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2616019@gndec.demo</t>
+          <t>2616019@gndec.test</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -4818,7 +4818,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2616020@gndec.demo</t>
+          <t>2616020@gndec.test</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -4845,7 +4845,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2616021@gndec.demo</t>
+          <t>2616021@gndec.test</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -4872,7 +4872,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2616022@gndec.demo</t>
+          <t>2616022@gndec.test</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2616023@gndec.demo</t>
+          <t>2616023@gndec.test</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -4926,7 +4926,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2616024@gndec.demo</t>
+          <t>2616024@gndec.test</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -4953,7 +4953,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2616025@gndec.demo</t>
+          <t>2616025@gndec.test</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -4980,7 +4980,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2616026@gndec.demo</t>
+          <t>2616026@gndec.test</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -5007,7 +5007,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2616027@gndec.demo</t>
+          <t>2616027@gndec.test</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2616028@gndec.demo</t>
+          <t>2616028@gndec.test</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -5061,7 +5061,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2616029@gndec.demo</t>
+          <t>2616029@gndec.test</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2616030@gndec.demo</t>
+          <t>2616030@gndec.test</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2616031@gndec.demo</t>
+          <t>2616031@gndec.test</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -5142,7 +5142,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2616032@gndec.demo</t>
+          <t>2616032@gndec.test</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -5169,7 +5169,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2616033@gndec.demo</t>
+          <t>2616033@gndec.test</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -5196,7 +5196,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2616034@gndec.demo</t>
+          <t>2616034@gndec.test</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -5223,7 +5223,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2616035@gndec.demo</t>
+          <t>2616035@gndec.test</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -5250,7 +5250,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2616036@gndec.demo</t>
+          <t>2616036@gndec.test</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -5277,7 +5277,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2616037@gndec.demo</t>
+          <t>2616037@gndec.test</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -5304,7 +5304,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2616038@gndec.demo</t>
+          <t>2616038@gndec.test</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2616039@gndec.demo</t>
+          <t>2616039@gndec.test</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -5358,7 +5358,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2616040@gndec.demo</t>
+          <t>2616040@gndec.test</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2616041@gndec.demo</t>
+          <t>2616041@gndec.test</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -5412,7 +5412,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2616042@gndec.demo</t>
+          <t>2616042@gndec.test</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -5439,7 +5439,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2616043@gndec.demo</t>
+          <t>2616043@gndec.test</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2616044@gndec.demo</t>
+          <t>2616044@gndec.test</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -5493,7 +5493,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2616045@gndec.demo</t>
+          <t>2616045@gndec.test</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2616046@gndec.demo</t>
+          <t>2616046@gndec.test</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5547,7 +5547,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2616047@gndec.demo</t>
+          <t>2616047@gndec.test</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2616048@gndec.demo</t>
+          <t>2616048@gndec.test</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5601,7 +5601,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2616049@gndec.demo</t>
+          <t>2616049@gndec.test</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5628,7 +5628,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2616050@gndec.demo</t>
+          <t>2616050@gndec.test</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5655,7 +5655,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2616051@gndec.demo</t>
+          <t>2616051@gndec.test</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -5682,7 +5682,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2616052@gndec.demo</t>
+          <t>2616052@gndec.test</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2616053@gndec.demo</t>
+          <t>2616053@gndec.test</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2616054@gndec.demo</t>
+          <t>2616054@gndec.test</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -5763,7 +5763,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2616055@gndec.demo</t>
+          <t>2616055@gndec.test</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -5790,7 +5790,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2616056@gndec.demo</t>
+          <t>2616056@gndec.test</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -5817,7 +5817,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2616057@gndec.demo</t>
+          <t>2616057@gndec.test</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -5844,7 +5844,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2616058@gndec.demo</t>
+          <t>2616058@gndec.test</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -5871,7 +5871,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2616059@gndec.demo</t>
+          <t>2616059@gndec.test</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -5898,7 +5898,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2616060@gndec.demo</t>
+          <t>2616060@gndec.test</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -5925,7 +5925,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2516001@gndec.demo</t>
+          <t>2516001@gndec.test</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2516002@gndec.demo</t>
+          <t>2516002@gndec.test</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -5979,7 +5979,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2516003@gndec.demo</t>
+          <t>2516003@gndec.test</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -6006,7 +6006,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2516004@gndec.demo</t>
+          <t>2516004@gndec.test</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -6033,7 +6033,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2516005@gndec.demo</t>
+          <t>2516005@gndec.test</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2516006@gndec.demo</t>
+          <t>2516006@gndec.test</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2516007@gndec.demo</t>
+          <t>2516007@gndec.test</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2516008@gndec.demo</t>
+          <t>2516008@gndec.test</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -6141,7 +6141,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2516009@gndec.demo</t>
+          <t>2516009@gndec.test</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -6168,7 +6168,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2516010@gndec.demo</t>
+          <t>2516010@gndec.test</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -6195,7 +6195,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2516011@gndec.demo</t>
+          <t>2516011@gndec.test</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -6222,7 +6222,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2516012@gndec.demo</t>
+          <t>2516012@gndec.test</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2516013@gndec.demo</t>
+          <t>2516013@gndec.test</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2516014@gndec.demo</t>
+          <t>2516014@gndec.test</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -6303,7 +6303,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2516015@gndec.demo</t>
+          <t>2516015@gndec.test</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2516016@gndec.demo</t>
+          <t>2516016@gndec.test</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -6357,7 +6357,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2516017@gndec.demo</t>
+          <t>2516017@gndec.test</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -6384,7 +6384,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2516018@gndec.demo</t>
+          <t>2516018@gndec.test</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -6411,7 +6411,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2516019@gndec.demo</t>
+          <t>2516019@gndec.test</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -6438,7 +6438,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2516020@gndec.demo</t>
+          <t>2516020@gndec.test</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -6465,7 +6465,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2516021@gndec.demo</t>
+          <t>2516021@gndec.test</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -6492,7 +6492,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2516022@gndec.demo</t>
+          <t>2516022@gndec.test</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2516023@gndec.demo</t>
+          <t>2516023@gndec.test</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -6546,7 +6546,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2516024@gndec.demo</t>
+          <t>2516024@gndec.test</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -6573,7 +6573,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2516025@gndec.demo</t>
+          <t>2516025@gndec.test</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -6600,7 +6600,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2516026@gndec.demo</t>
+          <t>2516026@gndec.test</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -6627,7 +6627,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2516027@gndec.demo</t>
+          <t>2516027@gndec.test</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -6654,7 +6654,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2516028@gndec.demo</t>
+          <t>2516028@gndec.test</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -6681,7 +6681,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2516029@gndec.demo</t>
+          <t>2516029@gndec.test</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -6708,7 +6708,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2516030@gndec.demo</t>
+          <t>2516030@gndec.test</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2516031@gndec.demo</t>
+          <t>2516031@gndec.test</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2516032@gndec.demo</t>
+          <t>2516032@gndec.test</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -6789,7 +6789,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2516033@gndec.demo</t>
+          <t>2516033@gndec.test</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -6816,7 +6816,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2516034@gndec.demo</t>
+          <t>2516034@gndec.test</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -6843,7 +6843,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2516035@gndec.demo</t>
+          <t>2516035@gndec.test</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -6870,7 +6870,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2516036@gndec.demo</t>
+          <t>2516036@gndec.test</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -6897,7 +6897,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2516037@gndec.demo</t>
+          <t>2516037@gndec.test</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -6924,7 +6924,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2516038@gndec.demo</t>
+          <t>2516038@gndec.test</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -6951,7 +6951,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2516039@gndec.demo</t>
+          <t>2516039@gndec.test</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -6978,7 +6978,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2516040@gndec.demo</t>
+          <t>2516040@gndec.test</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -7005,7 +7005,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2516041@gndec.demo</t>
+          <t>2516041@gndec.test</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -7032,7 +7032,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2516042@gndec.demo</t>
+          <t>2516042@gndec.test</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -7059,7 +7059,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2516043@gndec.demo</t>
+          <t>2516043@gndec.test</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -7086,7 +7086,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2516044@gndec.demo</t>
+          <t>2516044@gndec.test</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -7113,7 +7113,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2516045@gndec.demo</t>
+          <t>2516045@gndec.test</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2516046@gndec.demo</t>
+          <t>2516046@gndec.test</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -7167,7 +7167,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2516047@gndec.demo</t>
+          <t>2516047@gndec.test</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -7194,7 +7194,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2516048@gndec.demo</t>
+          <t>2516048@gndec.test</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -7221,7 +7221,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2516049@gndec.demo</t>
+          <t>2516049@gndec.test</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2516050@gndec.demo</t>
+          <t>2516050@gndec.test</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -7275,7 +7275,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2516051@gndec.demo</t>
+          <t>2516051@gndec.test</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2516052@gndec.demo</t>
+          <t>2516052@gndec.test</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -7329,7 +7329,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2516053@gndec.demo</t>
+          <t>2516053@gndec.test</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -7356,7 +7356,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2516054@gndec.demo</t>
+          <t>2516054@gndec.test</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2516055@gndec.demo</t>
+          <t>2516055@gndec.test</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -7410,7 +7410,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2516056@gndec.demo</t>
+          <t>2516056@gndec.test</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -7437,7 +7437,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2516057@gndec.demo</t>
+          <t>2516057@gndec.test</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2516058@gndec.demo</t>
+          <t>2516058@gndec.test</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2516059@gndec.demo</t>
+          <t>2516059@gndec.test</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -7518,7 +7518,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2516060@gndec.demo</t>
+          <t>2516060@gndec.test</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -7545,7 +7545,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2516061@gndec.demo</t>
+          <t>2516061@gndec.test</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -7572,7 +7572,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2516062@gndec.demo</t>
+          <t>2516062@gndec.test</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -7599,7 +7599,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2516063@gndec.demo</t>
+          <t>2516063@gndec.test</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -7626,7 +7626,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2516064@gndec.demo</t>
+          <t>2516064@gndec.test</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -7653,7 +7653,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2516065@gndec.demo</t>
+          <t>2516065@gndec.test</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -7680,7 +7680,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2516066@gndec.demo</t>
+          <t>2516066@gndec.test</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -7707,7 +7707,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2516067@gndec.demo</t>
+          <t>2516067@gndec.test</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -7734,7 +7734,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2516068@gndec.demo</t>
+          <t>2516068@gndec.test</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2516069@gndec.demo</t>
+          <t>2516069@gndec.test</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -7788,7 +7788,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2516070@gndec.demo</t>
+          <t>2516070@gndec.test</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2516071@gndec.demo</t>
+          <t>2516071@gndec.test</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -7842,7 +7842,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2516072@gndec.demo</t>
+          <t>2516072@gndec.test</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -7869,7 +7869,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2516073@gndec.demo</t>
+          <t>2516073@gndec.test</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -7896,7 +7896,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2516074@gndec.demo</t>
+          <t>2516074@gndec.test</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -7923,7 +7923,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2516075@gndec.demo</t>
+          <t>2516075@gndec.test</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -7950,7 +7950,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2516076@gndec.demo</t>
+          <t>2516076@gndec.test</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2516077@gndec.demo</t>
+          <t>2516077@gndec.test</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -8004,7 +8004,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2516078@gndec.demo</t>
+          <t>2516078@gndec.test</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -8031,7 +8031,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2516079@gndec.demo</t>
+          <t>2516079@gndec.test</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2516080@gndec.demo</t>
+          <t>2516080@gndec.test</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -8085,7 +8085,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2516081@gndec.demo</t>
+          <t>2516081@gndec.test</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2516082@gndec.demo</t>
+          <t>2516082@gndec.test</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -8139,7 +8139,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2516083@gndec.demo</t>
+          <t>2516083@gndec.test</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -8166,7 +8166,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2516084@gndec.demo</t>
+          <t>2516084@gndec.test</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -8193,7 +8193,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2516085@gndec.demo</t>
+          <t>2516085@gndec.test</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -8220,7 +8220,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2516086@gndec.demo</t>
+          <t>2516086@gndec.test</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -8247,7 +8247,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2516087@gndec.demo</t>
+          <t>2516087@gndec.test</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2516088@gndec.demo</t>
+          <t>2516088@gndec.test</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2516089@gndec.demo</t>
+          <t>2516089@gndec.test</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -8328,7 +8328,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2516090@gndec.demo</t>
+          <t>2516090@gndec.test</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -8355,7 +8355,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2516091@gndec.demo</t>
+          <t>2516091@gndec.test</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -8382,7 +8382,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2516092@gndec.demo</t>
+          <t>2516092@gndec.test</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -8409,7 +8409,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2516093@gndec.demo</t>
+          <t>2516093@gndec.test</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -8436,7 +8436,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2516094@gndec.demo</t>
+          <t>2516094@gndec.test</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -8463,7 +8463,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2516095@gndec.demo</t>
+          <t>2516095@gndec.test</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -8490,7 +8490,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2516096@gndec.demo</t>
+          <t>2516096@gndec.test</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -8517,7 +8517,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2516097@gndec.demo</t>
+          <t>2516097@gndec.test</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -8544,7 +8544,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2516098@gndec.demo</t>
+          <t>2516098@gndec.test</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -8571,7 +8571,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2516099@gndec.demo</t>
+          <t>2516099@gndec.test</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -8598,7 +8598,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2516100@gndec.demo</t>
+          <t>2516100@gndec.test</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -8625,7 +8625,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2516101@gndec.demo</t>
+          <t>2516101@gndec.test</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -8652,7 +8652,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2516102@gndec.demo</t>
+          <t>2516102@gndec.test</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -8679,7 +8679,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2516103@gndec.demo</t>
+          <t>2516103@gndec.test</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -8706,7 +8706,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2516104@gndec.demo</t>
+          <t>2516104@gndec.test</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2516105@gndec.demo</t>
+          <t>2516105@gndec.test</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -8760,7 +8760,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2516106@gndec.demo</t>
+          <t>2516106@gndec.test</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2516107@gndec.demo</t>
+          <t>2516107@gndec.test</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2516108@gndec.demo</t>
+          <t>2516108@gndec.test</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -8841,7 +8841,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2516109@gndec.demo</t>
+          <t>2516109@gndec.test</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -8868,7 +8868,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2516110@gndec.demo</t>
+          <t>2516110@gndec.test</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -8895,7 +8895,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2516111@gndec.demo</t>
+          <t>2516111@gndec.test</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2516112@gndec.demo</t>
+          <t>2516112@gndec.test</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -8949,7 +8949,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2516113@gndec.demo</t>
+          <t>2516113@gndec.test</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2516114@gndec.demo</t>
+          <t>2516114@gndec.test</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -9003,7 +9003,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2516115@gndec.demo</t>
+          <t>2516115@gndec.test</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2516116@gndec.demo</t>
+          <t>2516116@gndec.test</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -9057,7 +9057,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2516117@gndec.demo</t>
+          <t>2516117@gndec.test</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -9084,7 +9084,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2516118@gndec.demo</t>
+          <t>2516118@gndec.test</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -9111,7 +9111,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2416001@gndec.demo</t>
+          <t>2416001@gndec.test</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -9138,7 +9138,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2416002@gndec.demo</t>
+          <t>2416002@gndec.test</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -9165,7 +9165,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2416003@gndec.demo</t>
+          <t>2416003@gndec.test</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -9192,7 +9192,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2416004@gndec.demo</t>
+          <t>2416004@gndec.test</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -9219,7 +9219,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2416005@gndec.demo</t>
+          <t>2416005@gndec.test</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -9246,7 +9246,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2416006@gndec.demo</t>
+          <t>2416006@gndec.test</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -9273,7 +9273,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2416007@gndec.demo</t>
+          <t>2416007@gndec.test</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -9300,7 +9300,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2416008@gndec.demo</t>
+          <t>2416008@gndec.test</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -9327,7 +9327,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2416009@gndec.demo</t>
+          <t>2416009@gndec.test</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2416010@gndec.demo</t>
+          <t>2416010@gndec.test</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -9381,7 +9381,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2416011@gndec.demo</t>
+          <t>2416011@gndec.test</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -9408,7 +9408,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2416012@gndec.demo</t>
+          <t>2416012@gndec.test</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -9435,7 +9435,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2416013@gndec.demo</t>
+          <t>2416013@gndec.test</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -9462,7 +9462,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2416014@gndec.demo</t>
+          <t>2416014@gndec.test</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -9489,7 +9489,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2416015@gndec.demo</t>
+          <t>2416015@gndec.test</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -9516,7 +9516,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2416016@gndec.demo</t>
+          <t>2416016@gndec.test</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2416017@gndec.demo</t>
+          <t>2416017@gndec.test</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -9570,7 +9570,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2416018@gndec.demo</t>
+          <t>2416018@gndec.test</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -9597,7 +9597,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2416019@gndec.demo</t>
+          <t>2416019@gndec.test</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -9624,7 +9624,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2416020@gndec.demo</t>
+          <t>2416020@gndec.test</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -9651,7 +9651,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2416021@gndec.demo</t>
+          <t>2416021@gndec.test</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -9678,7 +9678,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2416022@gndec.demo</t>
+          <t>2416022@gndec.test</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2416023@gndec.demo</t>
+          <t>2416023@gndec.test</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -9732,7 +9732,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2416024@gndec.demo</t>
+          <t>2416024@gndec.test</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -9759,7 +9759,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>2416025@gndec.demo</t>
+          <t>2416025@gndec.test</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -9786,7 +9786,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>2416026@gndec.demo</t>
+          <t>2416026@gndec.test</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -9813,7 +9813,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>2416027@gndec.demo</t>
+          <t>2416027@gndec.test</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -9840,7 +9840,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>2416028@gndec.demo</t>
+          <t>2416028@gndec.test</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -9867,7 +9867,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>2416029@gndec.demo</t>
+          <t>2416029@gndec.test</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -9894,7 +9894,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>2416030@gndec.demo</t>
+          <t>2416030@gndec.test</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -9921,7 +9921,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>2416031@gndec.demo</t>
+          <t>2416031@gndec.test</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -9948,7 +9948,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>2416032@gndec.demo</t>
+          <t>2416032@gndec.test</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -9975,7 +9975,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>2416033@gndec.demo</t>
+          <t>2416033@gndec.test</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -10002,7 +10002,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>2416034@gndec.demo</t>
+          <t>2416034@gndec.test</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>2416035@gndec.demo</t>
+          <t>2416035@gndec.test</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
@@ -10056,7 +10056,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>2416036@gndec.demo</t>
+          <t>2416036@gndec.test</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -10083,7 +10083,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>2416037@gndec.demo</t>
+          <t>2416037@gndec.test</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -10110,7 +10110,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>2416038@gndec.demo</t>
+          <t>2416038@gndec.test</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -10137,7 +10137,7 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>2416039@gndec.demo</t>
+          <t>2416039@gndec.test</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>2416040@gndec.demo</t>
+          <t>2416040@gndec.test</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
@@ -10191,7 +10191,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>2416041@gndec.demo</t>
+          <t>2416041@gndec.test</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
@@ -10218,7 +10218,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>2416042@gndec.demo</t>
+          <t>2416042@gndec.test</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
@@ -10245,7 +10245,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>2416043@gndec.demo</t>
+          <t>2416043@gndec.test</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
@@ -10272,7 +10272,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>2416044@gndec.demo</t>
+          <t>2416044@gndec.test</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
@@ -10299,7 +10299,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>2416045@gndec.demo</t>
+          <t>2416045@gndec.test</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -10326,7 +10326,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>2416046@gndec.demo</t>
+          <t>2416046@gndec.test</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
@@ -10353,7 +10353,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>2416047@gndec.demo</t>
+          <t>2416047@gndec.test</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
@@ -10380,7 +10380,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>2416048@gndec.demo</t>
+          <t>2416048@gndec.test</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
@@ -10407,7 +10407,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>2416049@gndec.demo</t>
+          <t>2416049@gndec.test</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
@@ -10434,7 +10434,7 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>2416050@gndec.demo</t>
+          <t>2416050@gndec.test</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
@@ -10461,7 +10461,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>2416051@gndec.demo</t>
+          <t>2416051@gndec.test</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
@@ -10488,7 +10488,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>2416052@gndec.demo</t>
+          <t>2416052@gndec.test</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -10515,7 +10515,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>2416053@gndec.demo</t>
+          <t>2416053@gndec.test</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
@@ -10542,7 +10542,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>2416054@gndec.demo</t>
+          <t>2416054@gndec.test</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -10569,7 +10569,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>2416055@gndec.demo</t>
+          <t>2416055@gndec.test</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -10596,7 +10596,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>2416056@gndec.demo</t>
+          <t>2416056@gndec.test</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -10623,7 +10623,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>2416057@gndec.demo</t>
+          <t>2416057@gndec.test</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -10650,7 +10650,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>2416058@gndec.demo</t>
+          <t>2416058@gndec.test</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -10677,7 +10677,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>2416059@gndec.demo</t>
+          <t>2416059@gndec.test</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -10704,7 +10704,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>2416060@gndec.demo</t>
+          <t>2416060@gndec.test</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -10731,7 +10731,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>2416061@gndec.demo</t>
+          <t>2416061@gndec.test</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>2416062@gndec.demo</t>
+          <t>2416062@gndec.test</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -10785,7 +10785,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>2416063@gndec.demo</t>
+          <t>2416063@gndec.test</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -10812,7 +10812,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>2416064@gndec.demo</t>
+          <t>2416064@gndec.test</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>2416065@gndec.demo</t>
+          <t>2416065@gndec.test</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -10866,7 +10866,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>2416066@gndec.demo</t>
+          <t>2416066@gndec.test</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>2416067@gndec.demo</t>
+          <t>2416067@gndec.test</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -10920,7 +10920,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>2416068@gndec.demo</t>
+          <t>2416068@gndec.test</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -10947,7 +10947,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>2416069@gndec.demo</t>
+          <t>2416069@gndec.test</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -10974,7 +10974,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>2416070@gndec.demo</t>
+          <t>2416070@gndec.test</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -11001,7 +11001,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>2416071@gndec.demo</t>
+          <t>2416071@gndec.test</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -11028,7 +11028,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>2416072@gndec.demo</t>
+          <t>2416072@gndec.test</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -11055,7 +11055,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>2416073@gndec.demo</t>
+          <t>2416073@gndec.test</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>2416074@gndec.demo</t>
+          <t>2416074@gndec.test</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -11109,7 +11109,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>2416075@gndec.demo</t>
+          <t>2416075@gndec.test</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -11136,7 +11136,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>2416076@gndec.demo</t>
+          <t>2416076@gndec.test</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -11163,7 +11163,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>2416077@gndec.demo</t>
+          <t>2416077@gndec.test</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -11190,7 +11190,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2416078@gndec.demo</t>
+          <t>2416078@gndec.test</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -11217,7 +11217,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2416079@gndec.demo</t>
+          <t>2416079@gndec.test</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -11244,7 +11244,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>2416080@gndec.demo</t>
+          <t>2416080@gndec.test</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -11271,7 +11271,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>2416081@gndec.demo</t>
+          <t>2416081@gndec.test</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -11298,7 +11298,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2416082@gndec.demo</t>
+          <t>2416082@gndec.test</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -11325,7 +11325,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2416083@gndec.demo</t>
+          <t>2416083@gndec.test</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -11352,7 +11352,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2416084@gndec.demo</t>
+          <t>2416084@gndec.test</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -11379,7 +11379,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2416085@gndec.demo</t>
+          <t>2416085@gndec.test</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -11406,7 +11406,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2416086@gndec.demo</t>
+          <t>2416086@gndec.test</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -11433,7 +11433,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>2416087@gndec.demo</t>
+          <t>2416087@gndec.test</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -11460,7 +11460,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>2416088@gndec.demo</t>
+          <t>2416088@gndec.test</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>2416089@gndec.demo</t>
+          <t>2416089@gndec.test</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
@@ -11514,7 +11514,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>2416090@gndec.demo</t>
+          <t>2416090@gndec.test</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -11541,7 +11541,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>2416091@gndec.demo</t>
+          <t>2416091@gndec.test</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -11568,7 +11568,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>2416092@gndec.demo</t>
+          <t>2416092@gndec.test</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -11595,7 +11595,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>2416093@gndec.demo</t>
+          <t>2416093@gndec.test</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -11622,7 +11622,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>2416094@gndec.demo</t>
+          <t>2416094@gndec.test</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -11649,7 +11649,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>2416095@gndec.demo</t>
+          <t>2416095@gndec.test</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -11676,7 +11676,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2416096@gndec.demo</t>
+          <t>2416096@gndec.test</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -11703,7 +11703,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>2416097@gndec.demo</t>
+          <t>2416097@gndec.test</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -11730,7 +11730,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>2416098@gndec.demo</t>
+          <t>2416098@gndec.test</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -11757,7 +11757,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>2416099@gndec.demo</t>
+          <t>2416099@gndec.test</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -11784,7 +11784,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>2416100@gndec.demo</t>
+          <t>2416100@gndec.test</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -11811,7 +11811,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>2416101@gndec.demo</t>
+          <t>2416101@gndec.test</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -11838,7 +11838,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>2416102@gndec.demo</t>
+          <t>2416102@gndec.test</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>2416103@gndec.demo</t>
+          <t>2416103@gndec.test</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -11892,7 +11892,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>2416104@gndec.demo</t>
+          <t>2416104@gndec.test</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -11919,7 +11919,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2416105@gndec.demo</t>
+          <t>2416105@gndec.test</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -11946,7 +11946,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2416106@gndec.demo</t>
+          <t>2416106@gndec.test</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -11973,7 +11973,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2416107@gndec.demo</t>
+          <t>2416107@gndec.test</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -12000,7 +12000,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>2416108@gndec.demo</t>
+          <t>2416108@gndec.test</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -12027,7 +12027,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>2416109@gndec.demo</t>
+          <t>2416109@gndec.test</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -12054,7 +12054,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>2416110@gndec.demo</t>
+          <t>2416110@gndec.test</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -12081,7 +12081,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>2416111@gndec.demo</t>
+          <t>2416111@gndec.test</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
@@ -12108,7 +12108,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>2416112@gndec.demo</t>
+          <t>2416112@gndec.test</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
@@ -12135,7 +12135,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>2416113@gndec.demo</t>
+          <t>2416113@gndec.test</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
@@ -12162,7 +12162,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>2416114@gndec.demo</t>
+          <t>2416114@gndec.test</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
@@ -12189,7 +12189,7 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>2416115@gndec.demo</t>
+          <t>2416115@gndec.test</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
@@ -12216,7 +12216,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>2416116@gndec.demo</t>
+          <t>2416116@gndec.test</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
@@ -12243,7 +12243,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>2416117@gndec.demo</t>
+          <t>2416117@gndec.test</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
@@ -12270,7 +12270,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>2416118@gndec.demo</t>
+          <t>2416118@gndec.test</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
@@ -12297,7 +12297,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>2316001@gndec.demo</t>
+          <t>2316001@gndec.test</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
@@ -12324,7 +12324,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>2316002@gndec.demo</t>
+          <t>2316002@gndec.test</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
@@ -12351,7 +12351,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>2316003@gndec.demo</t>
+          <t>2316003@gndec.test</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
@@ -12378,7 +12378,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>2316004@gndec.demo</t>
+          <t>2316004@gndec.test</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
@@ -12405,7 +12405,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>2316005@gndec.demo</t>
+          <t>2316005@gndec.test</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
@@ -12432,7 +12432,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>2316006@gndec.demo</t>
+          <t>2316006@gndec.test</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
@@ -12459,7 +12459,7 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>2316007@gndec.demo</t>
+          <t>2316007@gndec.test</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>2316008@gndec.demo</t>
+          <t>2316008@gndec.test</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
@@ -12513,7 +12513,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>2316009@gndec.demo</t>
+          <t>2316009@gndec.test</t>
         </is>
       </c>
       <c r="D306" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>2316010@gndec.demo</t>
+          <t>2316010@gndec.test</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
@@ -12567,7 +12567,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>2316011@gndec.demo</t>
+          <t>2316011@gndec.test</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
@@ -12594,7 +12594,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>2316012@gndec.demo</t>
+          <t>2316012@gndec.test</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
@@ -12621,7 +12621,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>2316013@gndec.demo</t>
+          <t>2316013@gndec.test</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
@@ -12648,7 +12648,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>2316014@gndec.demo</t>
+          <t>2316014@gndec.test</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
@@ -12675,7 +12675,7 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>2316015@gndec.demo</t>
+          <t>2316015@gndec.test</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
@@ -12702,7 +12702,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>2316016@gndec.demo</t>
+          <t>2316016@gndec.test</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
@@ -12729,7 +12729,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>2316017@gndec.demo</t>
+          <t>2316017@gndec.test</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
@@ -12756,7 +12756,7 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>2316018@gndec.demo</t>
+          <t>2316018@gndec.test</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
@@ -12783,7 +12783,7 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>2316019@gndec.demo</t>
+          <t>2316019@gndec.test</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
@@ -12810,7 +12810,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>2316020@gndec.demo</t>
+          <t>2316020@gndec.test</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
@@ -12837,7 +12837,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>2316021@gndec.demo</t>
+          <t>2316021@gndec.test</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
@@ -12864,7 +12864,7 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>2316022@gndec.demo</t>
+          <t>2316022@gndec.test</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>2316023@gndec.demo</t>
+          <t>2316023@gndec.test</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
@@ -12918,7 +12918,7 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>2316024@gndec.demo</t>
+          <t>2316024@gndec.test</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
@@ -12945,7 +12945,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>2316025@gndec.demo</t>
+          <t>2316025@gndec.test</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
@@ -12972,7 +12972,7 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>2316026@gndec.demo</t>
+          <t>2316026@gndec.test</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
@@ -12999,7 +12999,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>2316027@gndec.demo</t>
+          <t>2316027@gndec.test</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
@@ -13026,7 +13026,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>2316028@gndec.demo</t>
+          <t>2316028@gndec.test</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
@@ -13053,7 +13053,7 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>2316029@gndec.demo</t>
+          <t>2316029@gndec.test</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
@@ -13080,7 +13080,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>2316030@gndec.demo</t>
+          <t>2316030@gndec.test</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
@@ -13107,7 +13107,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>2316031@gndec.demo</t>
+          <t>2316031@gndec.test</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
@@ -13134,7 +13134,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>2316032@gndec.demo</t>
+          <t>2316032@gndec.test</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
@@ -13161,7 +13161,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>2316033@gndec.demo</t>
+          <t>2316033@gndec.test</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
@@ -13188,7 +13188,7 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>2316034@gndec.demo</t>
+          <t>2316034@gndec.test</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>2316035@gndec.demo</t>
+          <t>2316035@gndec.test</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
@@ -13242,7 +13242,7 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>2316036@gndec.demo</t>
+          <t>2316036@gndec.test</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>2316037@gndec.demo</t>
+          <t>2316037@gndec.test</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
@@ -13296,7 +13296,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>2316038@gndec.demo</t>
+          <t>2316038@gndec.test</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
@@ -13323,7 +13323,7 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>2316039@gndec.demo</t>
+          <t>2316039@gndec.test</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
@@ -13350,7 +13350,7 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>2316040@gndec.demo</t>
+          <t>2316040@gndec.test</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
@@ -13377,7 +13377,7 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>2316041@gndec.demo</t>
+          <t>2316041@gndec.test</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>2316042@gndec.demo</t>
+          <t>2316042@gndec.test</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
@@ -13431,7 +13431,7 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>2316043@gndec.demo</t>
+          <t>2316043@gndec.test</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
@@ -13458,7 +13458,7 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>2316044@gndec.demo</t>
+          <t>2316044@gndec.test</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
@@ -13485,7 +13485,7 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>2316045@gndec.demo</t>
+          <t>2316045@gndec.test</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
@@ -13512,7 +13512,7 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>2316046@gndec.demo</t>
+          <t>2316046@gndec.test</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
@@ -13539,7 +13539,7 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>2316047@gndec.demo</t>
+          <t>2316047@gndec.test</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
@@ -13566,7 +13566,7 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>2316048@gndec.demo</t>
+          <t>2316048@gndec.test</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
@@ -13593,7 +13593,7 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>2316049@gndec.demo</t>
+          <t>2316049@gndec.test</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
@@ -13620,7 +13620,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>2316050@gndec.demo</t>
+          <t>2316050@gndec.test</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
@@ -13647,7 +13647,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>2316051@gndec.demo</t>
+          <t>2316051@gndec.test</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
@@ -13674,7 +13674,7 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>2316052@gndec.demo</t>
+          <t>2316052@gndec.test</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
@@ -13701,7 +13701,7 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>2316053@gndec.demo</t>
+          <t>2316053@gndec.test</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
@@ -13728,7 +13728,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>2316054@gndec.demo</t>
+          <t>2316054@gndec.test</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
@@ -13755,7 +13755,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>2316055@gndec.demo</t>
+          <t>2316055@gndec.test</t>
         </is>
       </c>
       <c r="D352" t="inlineStr">
@@ -13782,7 +13782,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>2316056@gndec.demo</t>
+          <t>2316056@gndec.test</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
@@ -13809,7 +13809,7 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>2316057@gndec.demo</t>
+          <t>2316057@gndec.test</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
@@ -13836,7 +13836,7 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>2316058@gndec.demo</t>
+          <t>2316058@gndec.test</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
@@ -13863,7 +13863,7 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>2316059@gndec.demo</t>
+          <t>2316059@gndec.test</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
@@ -13890,7 +13890,7 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>2316060@gndec.demo</t>
+          <t>2316060@gndec.test</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>2316061@gndec.demo</t>
+          <t>2316061@gndec.test</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
@@ -13944,7 +13944,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>2316062@gndec.demo</t>
+          <t>2316062@gndec.test</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
@@ -13971,7 +13971,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>2316063@gndec.demo</t>
+          <t>2316063@gndec.test</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
@@ -13998,7 +13998,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>2316064@gndec.demo</t>
+          <t>2316064@gndec.test</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
@@ -14025,7 +14025,7 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>2316065@gndec.demo</t>
+          <t>2316065@gndec.test</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
@@ -14052,7 +14052,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>2316066@gndec.demo</t>
+          <t>2316066@gndec.test</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
@@ -14079,7 +14079,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>2316067@gndec.demo</t>
+          <t>2316067@gndec.test</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
@@ -14106,7 +14106,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>2316068@gndec.demo</t>
+          <t>2316068@gndec.test</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
@@ -14133,7 +14133,7 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>2316069@gndec.demo</t>
+          <t>2316069@gndec.test</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>2316070@gndec.demo</t>
+          <t>2316070@gndec.test</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
@@ -14187,7 +14187,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>2316071@gndec.demo</t>
+          <t>2316071@gndec.test</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
@@ -14214,7 +14214,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>2316072@gndec.demo</t>
+          <t>2316072@gndec.test</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
@@ -14241,7 +14241,7 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>2316073@gndec.demo</t>
+          <t>2316073@gndec.test</t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
@@ -14268,7 +14268,7 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>2316074@gndec.demo</t>
+          <t>2316074@gndec.test</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
@@ -14295,7 +14295,7 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>2316075@gndec.demo</t>
+          <t>2316075@gndec.test</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
@@ -14322,7 +14322,7 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>2316076@gndec.demo</t>
+          <t>2316076@gndec.test</t>
         </is>
       </c>
       <c r="D373" t="inlineStr">
@@ -14349,7 +14349,7 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>2316077@gndec.demo</t>
+          <t>2316077@gndec.test</t>
         </is>
       </c>
       <c r="D374" t="inlineStr">
@@ -14376,7 +14376,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>2316078@gndec.demo</t>
+          <t>2316078@gndec.test</t>
         </is>
       </c>
       <c r="D375" t="inlineStr">
@@ -14403,7 +14403,7 @@
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>2316079@gndec.demo</t>
+          <t>2316079@gndec.test</t>
         </is>
       </c>
       <c r="D376" t="inlineStr">
@@ -14430,7 +14430,7 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>2316080@gndec.demo</t>
+          <t>2316080@gndec.test</t>
         </is>
       </c>
       <c r="D377" t="inlineStr">
@@ -14457,7 +14457,7 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>2316081@gndec.demo</t>
+          <t>2316081@gndec.test</t>
         </is>
       </c>
       <c r="D378" t="inlineStr">
@@ -14484,7 +14484,7 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>2316082@gndec.demo</t>
+          <t>2316082@gndec.test</t>
         </is>
       </c>
       <c r="D379" t="inlineStr">
@@ -14511,7 +14511,7 @@
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>2316083@gndec.demo</t>
+          <t>2316083@gndec.test</t>
         </is>
       </c>
       <c r="D380" t="inlineStr">
@@ -14538,7 +14538,7 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>2316084@gndec.demo</t>
+          <t>2316084@gndec.test</t>
         </is>
       </c>
       <c r="D381" t="inlineStr">
@@ -14565,7 +14565,7 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>2316085@gndec.demo</t>
+          <t>2316085@gndec.test</t>
         </is>
       </c>
       <c r="D382" t="inlineStr">
@@ -14592,7 +14592,7 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>2316086@gndec.demo</t>
+          <t>2316086@gndec.test</t>
         </is>
       </c>
       <c r="D383" t="inlineStr">
@@ -14619,7 +14619,7 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>2316087@gndec.demo</t>
+          <t>2316087@gndec.test</t>
         </is>
       </c>
       <c r="D384" t="inlineStr">
@@ -14646,7 +14646,7 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>2316088@gndec.demo</t>
+          <t>2316088@gndec.test</t>
         </is>
       </c>
       <c r="D385" t="inlineStr">
@@ -14673,7 +14673,7 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>2316089@gndec.demo</t>
+          <t>2316089@gndec.test</t>
         </is>
       </c>
       <c r="D386" t="inlineStr">
@@ -14700,7 +14700,7 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>2316090@gndec.demo</t>
+          <t>2316090@gndec.test</t>
         </is>
       </c>
       <c r="D387" t="inlineStr">
@@ -14727,7 +14727,7 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>2316091@gndec.demo</t>
+          <t>2316091@gndec.test</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
@@ -14754,7 +14754,7 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>2316092@gndec.demo</t>
+          <t>2316092@gndec.test</t>
         </is>
       </c>
       <c r="D389" t="inlineStr">
@@ -14781,7 +14781,7 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>2316093@gndec.demo</t>
+          <t>2316093@gndec.test</t>
         </is>
       </c>
       <c r="D390" t="inlineStr">
@@ -14808,7 +14808,7 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>2316094@gndec.demo</t>
+          <t>2316094@gndec.test</t>
         </is>
       </c>
       <c r="D391" t="inlineStr">
@@ -14835,7 +14835,7 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>2316095@gndec.demo</t>
+          <t>2316095@gndec.test</t>
         </is>
       </c>
       <c r="D392" t="inlineStr">
@@ -14862,7 +14862,7 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>2316096@gndec.demo</t>
+          <t>2316096@gndec.test</t>
         </is>
       </c>
       <c r="D393" t="inlineStr">
@@ -14889,7 +14889,7 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>2316097@gndec.demo</t>
+          <t>2316097@gndec.test</t>
         </is>
       </c>
       <c r="D394" t="inlineStr">
@@ -14916,7 +14916,7 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>2316098@gndec.demo</t>
+          <t>2316098@gndec.test</t>
         </is>
       </c>
       <c r="D395" t="inlineStr">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>2316099@gndec.demo</t>
+          <t>2316099@gndec.test</t>
         </is>
       </c>
       <c r="D396" t="inlineStr">
@@ -14970,7 +14970,7 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>2316100@gndec.demo</t>
+          <t>2316100@gndec.test</t>
         </is>
       </c>
       <c r="D397" t="inlineStr">
@@ -14997,7 +14997,7 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>2316101@gndec.demo</t>
+          <t>2316101@gndec.test</t>
         </is>
       </c>
       <c r="D398" t="inlineStr">
@@ -15024,7 +15024,7 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>2316102@gndec.demo</t>
+          <t>2316102@gndec.test</t>
         </is>
       </c>
       <c r="D399" t="inlineStr">
@@ -15051,7 +15051,7 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>2316103@gndec.demo</t>
+          <t>2316103@gndec.test</t>
         </is>
       </c>
       <c r="D400" t="inlineStr">
@@ -15078,7 +15078,7 @@
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>2316104@gndec.demo</t>
+          <t>2316104@gndec.test</t>
         </is>
       </c>
       <c r="D401" t="inlineStr">
@@ -15105,7 +15105,7 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>2316105@gndec.demo</t>
+          <t>2316105@gndec.test</t>
         </is>
       </c>
       <c r="D402" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>2316106@gndec.demo</t>
+          <t>2316106@gndec.test</t>
         </is>
       </c>
       <c r="D403" t="inlineStr">
@@ -15159,7 +15159,7 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>2316107@gndec.demo</t>
+          <t>2316107@gndec.test</t>
         </is>
       </c>
       <c r="D404" t="inlineStr">
@@ -15186,7 +15186,7 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>2316108@gndec.demo</t>
+          <t>2316108@gndec.test</t>
         </is>
       </c>
       <c r="D405" t="inlineStr">
@@ -15213,7 +15213,7 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>2316109@gndec.demo</t>
+          <t>2316109@gndec.test</t>
         </is>
       </c>
       <c r="D406" t="inlineStr">
@@ -15240,7 +15240,7 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>2316110@gndec.demo</t>
+          <t>2316110@gndec.test</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
@@ -15267,7 +15267,7 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>2316111@gndec.demo</t>
+          <t>2316111@gndec.test</t>
         </is>
       </c>
       <c r="D408" t="inlineStr">
@@ -15294,7 +15294,7 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>2316112@gndec.demo</t>
+          <t>2316112@gndec.test</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
@@ -15321,7 +15321,7 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>2316113@gndec.demo</t>
+          <t>2316113@gndec.test</t>
         </is>
       </c>
       <c r="D410" t="inlineStr">
@@ -15348,7 +15348,7 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>2316114@gndec.demo</t>
+          <t>2316114@gndec.test</t>
         </is>
       </c>
       <c r="D411" t="inlineStr">
@@ -15375,7 +15375,7 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>2316115@gndec.demo</t>
+          <t>2316115@gndec.test</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
@@ -15402,7 +15402,7 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>2316116@gndec.demo</t>
+          <t>2316116@gndec.test</t>
         </is>
       </c>
       <c r="D413" t="inlineStr">
@@ -15429,7 +15429,7 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>2316117@gndec.demo</t>
+          <t>2316117@gndec.test</t>
         </is>
       </c>
       <c r="D414" t="inlineStr">
@@ -15456,7 +15456,7 @@
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>2316118@gndec.demo</t>
+          <t>2316118@gndec.test</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">

</xml_diff>